<commit_message>
update implementing column of values and unit
</commit_message>
<xml_diff>
--- a/data/final/bplan_samples/annotation/filled_company_templates/test_filled_annotation.xlsx
+++ b/data/final/bplan_samples/annotation/filled_company_templates/test_filled_annotation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>id</t>
   </si>
@@ -79,10 +79,22 @@
     <t xml:space="preserve">695_0.jpg</t>
   </si>
   <si>
-    <t xml:space="preserve">grz</t>
+    <t xml:space="preserve">grz_value</t>
   </si>
   <si>
-    <t xml:space="preserve">gfz</t>
+    <t xml:space="preserve">gfz_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eg_fok_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eg_fok_unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eg_fok</t>
   </si>
   <si>
     <t xml:space="preserve">807_0.jpg</t>
@@ -497,9 +509,7 @@
       <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>0.35</v>
-      </c>
+      <c r="D2" s="2"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="4"/>
@@ -515,9 +525,7 @@
       <c r="C3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>0.35</v>
-      </c>
+      <c r="D3" s="2"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="4"/>
@@ -525,17 +533,15 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>807</v>
+        <v>695</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>0.6</v>
-      </c>
+      <c r="D4" s="2"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="4"/>
@@ -543,17 +549,15 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>807</v>
+        <v>695</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="D5" s="2"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
@@ -561,17 +565,15 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="n">
-        <v>904</v>
+        <v>695</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>0.6</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
@@ -579,17 +581,15 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="n">
-        <v>904</v>
+        <v>695</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>2</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="4"/>
@@ -597,15 +597,17 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="2" t="n">
-        <v>904</v>
+        <v>807</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" s="2" t="n">
+        <v>0.6</v>
+      </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="4"/>
@@ -613,15 +615,17 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="2" t="n">
-        <v>904</v>
+        <v>807</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="2"/>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="4"/>
@@ -629,13 +633,13 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="2" t="n">
-        <v>904</v>
+        <v>807</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
@@ -645,13 +649,13 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="2" t="n">
-        <v>904</v>
+        <v>807</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
@@ -661,13 +665,13 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="2" t="n">
-        <v>904</v>
+        <v>807</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="3"/>
@@ -677,13 +681,13 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="2" t="n">
-        <v>904</v>
+        <v>807</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="3"/>
@@ -732,10 +736,10 @@
         <v>904</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="3"/>
@@ -748,10 +752,10 @@
         <v>904</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="3"/>
@@ -764,10 +768,10 @@
         <v>904</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="3"/>
@@ -780,10 +784,10 @@
         <v>904</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="3"/>
@@ -796,7 +800,7 @@
         <v>904</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>21</v>
@@ -812,7 +816,7 @@
         <v>904</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>22</v>
@@ -828,10 +832,10 @@
         <v>904</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="3"/>
@@ -844,10 +848,10 @@
         <v>904</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="3"/>
@@ -856,9 +860,15 @@
       <c r="H23" s="1"/>
     </row>
     <row r="24" ht="12.5" customHeight="1">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
+      <c r="A24" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D24" s="2"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -866,9 +876,15 @@
       <c r="H24" s="1"/>
     </row>
     <row r="25" ht="12.5" customHeight="1">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
+      <c r="A25" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D25" s="2"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -876,9 +892,15 @@
       <c r="H25" s="1"/>
     </row>
     <row r="26" ht="12.5" customHeight="1">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
+      <c r="A26" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D26" s="2"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -886,9 +908,15 @@
       <c r="H26" s="1"/>
     </row>
     <row r="27" ht="12.5" customHeight="1">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="A27" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D27" s="2"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
@@ -896,9 +924,15 @@
       <c r="H27" s="1"/>
     </row>
     <row r="28" ht="12.5" customHeight="1">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="A28" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D28" s="2"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
@@ -906,9 +940,15 @@
       <c r="H28" s="1"/>
     </row>
     <row r="29" ht="12.5" customHeight="1">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
+      <c r="A29" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D29" s="2"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
@@ -916,9 +956,15 @@
       <c r="H29" s="1"/>
     </row>
     <row r="30" ht="12.5" customHeight="1">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
+      <c r="A30" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D30" s="2"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
@@ -926,9 +972,15 @@
       <c r="H30" s="1"/>
     </row>
     <row r="31" ht="12.5" customHeight="1">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
+      <c r="A31" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D31" s="2"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -936,9 +988,15 @@
       <c r="H31" s="1"/>
     </row>
     <row r="32" ht="12.5" customHeight="1">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
+      <c r="A32" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D32" s="2"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -946,9 +1004,15 @@
       <c r="H32" s="1"/>
     </row>
     <row r="33" ht="12.5" customHeight="1">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
+      <c r="A33" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D33" s="2"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
@@ -956,9 +1020,15 @@
       <c r="H33" s="1"/>
     </row>
     <row r="34" ht="12.5" customHeight="1">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
+      <c r="A34" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D34" s="2"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -966,9 +1036,15 @@
       <c r="H34" s="1"/>
     </row>
     <row r="35" ht="12.5" customHeight="1">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
+      <c r="A35" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D35" s="2"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
@@ -976,9 +1052,15 @@
       <c r="H35" s="1"/>
     </row>
     <row r="36" ht="12.5" customHeight="1">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
+      <c r="A36" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D36" s="2"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -986,9 +1068,15 @@
       <c r="H36" s="1"/>
     </row>
     <row r="37" ht="12.5" customHeight="1">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
+      <c r="A37" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D37" s="2"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -996,29 +1084,51 @@
       <c r="H37" s="1"/>
     </row>
     <row r="38" ht="12.5" customHeight="1">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="A38" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>0.6</v>
+      </c>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
       <c r="G38" s="4"/>
       <c r="H38" s="1"/>
     </row>
     <row r="39" ht="12.5" customHeight="1">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="A39" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
       <c r="G39" s="4"/>
       <c r="H39" s="1"/>
     </row>
     <row r="40" ht="12.5" customHeight="1">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
+      <c r="A40" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D40" s="2"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -1026,9 +1136,15 @@
       <c r="H40" s="1"/>
     </row>
     <row r="41" ht="12.5" customHeight="1">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
+      <c r="A41" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D41" s="2"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -1036,9 +1152,15 @@
       <c r="H41" s="1"/>
     </row>
     <row r="42" ht="12.5" customHeight="1">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
+      <c r="A42" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D42" s="2"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
@@ -1046,9 +1168,15 @@
       <c r="H42" s="1"/>
     </row>
     <row r="43" ht="12.5" customHeight="1">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
+      <c r="A43" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D43" s="2"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -1056,9 +1184,15 @@
       <c r="H43" s="1"/>
     </row>
     <row r="44" ht="12.5" customHeight="1">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
+      <c r="A44" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D44" s="2"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
@@ -1066,9 +1200,15 @@
       <c r="H44" s="1"/>
     </row>
     <row r="45" ht="12.5" customHeight="1">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
+      <c r="A45" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D45" s="2"/>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
@@ -1076,9 +1216,15 @@
       <c r="H45" s="1"/>
     </row>
     <row r="46" ht="12.5" customHeight="1">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
+      <c r="A46" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D46" s="2"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
@@ -1086,9 +1232,15 @@
       <c r="H46" s="1"/>
     </row>
     <row r="47" ht="12.5" customHeight="1">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
+      <c r="A47" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D47" s="2"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
@@ -1096,9 +1248,15 @@
       <c r="H47" s="1"/>
     </row>
     <row r="48" ht="12.5" customHeight="1">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
+      <c r="A48" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D48" s="2"/>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
@@ -1106,9 +1264,15 @@
       <c r="H48" s="1"/>
     </row>
     <row r="49" ht="12.5" customHeight="1">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
+      <c r="A49" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D49" s="2"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
@@ -1116,9 +1280,15 @@
       <c r="H49" s="1"/>
     </row>
     <row r="50" ht="12.5" customHeight="1">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
+      <c r="A50" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D50" s="2"/>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -1126,9 +1296,15 @@
       <c r="H50" s="1"/>
     </row>
     <row r="51" ht="12.5" customHeight="1">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
+      <c r="A51" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D51" s="2"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -1136,9 +1312,15 @@
       <c r="H51" s="1"/>
     </row>
     <row r="52" ht="12.5" customHeight="1">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
+      <c r="A52" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D52" s="2"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
@@ -1146,9 +1328,15 @@
       <c r="H52" s="1"/>
     </row>
     <row r="53" ht="12.5" customHeight="1">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
+      <c r="A53" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D53" s="2"/>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -1156,9 +1344,15 @@
       <c r="H53" s="1"/>
     </row>
     <row r="54" ht="12.5" customHeight="1">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
+      <c r="A54" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D54" s="2"/>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
@@ -1166,9 +1360,15 @@
       <c r="H54" s="1"/>
     </row>
     <row r="55" ht="12.5" customHeight="1">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
+      <c r="A55" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D55" s="2"/>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
@@ -1176,9 +1376,15 @@
       <c r="H55" s="1"/>
     </row>
     <row r="56" ht="12.5" customHeight="1">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
+      <c r="A56" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D56" s="2"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
@@ -1186,9 +1392,15 @@
       <c r="H56" s="1"/>
     </row>
     <row r="57" ht="12.5" customHeight="1">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
+      <c r="A57" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D57" s="2"/>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
@@ -1196,9 +1408,15 @@
       <c r="H57" s="1"/>
     </row>
     <row r="58" ht="12.5" customHeight="1">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
+      <c r="A58" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D58" s="2"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
@@ -1206,9 +1424,15 @@
       <c r="H58" s="1"/>
     </row>
     <row r="59" ht="12.5" customHeight="1">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
+      <c r="A59" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D59" s="2"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
@@ -1216,9 +1440,15 @@
       <c r="H59" s="1"/>
     </row>
     <row r="60" ht="12.5" customHeight="1">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
+      <c r="A60" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D60" s="2"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
@@ -1226,9 +1456,15 @@
       <c r="H60" s="1"/>
     </row>
     <row r="61" ht="12.5" customHeight="1">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
+      <c r="A61" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D61" s="2"/>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
@@ -1236,9 +1472,15 @@
       <c r="H61" s="1"/>
     </row>
     <row r="62" ht="12.5" customHeight="1">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
+      <c r="A62" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="D62" s="2"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
@@ -1246,9 +1488,15 @@
       <c r="H62" s="1"/>
     </row>
     <row r="63" ht="12.5" customHeight="1">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
+      <c r="A63" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="D63" s="2"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
@@ -1256,9 +1504,15 @@
       <c r="H63" s="1"/>
     </row>
     <row r="64" ht="12.5" customHeight="1">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
+      <c r="A64" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D64" s="2"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
@@ -1266,9 +1520,15 @@
       <c r="H64" s="1"/>
     </row>
     <row r="65" ht="12.5" customHeight="1">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
+      <c r="A65" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="D65" s="2"/>
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
@@ -1276,9 +1536,15 @@
       <c r="H65" s="1"/>
     </row>
     <row r="66" ht="12.5" customHeight="1">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
+      <c r="A66" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D66" s="2"/>
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
@@ -1286,9 +1552,15 @@
       <c r="H66" s="1"/>
     </row>
     <row r="67" ht="12.5" customHeight="1">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
+      <c r="A67" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="D67" s="2"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>

</xml_diff>

<commit_message>
get bp text parsed from vm
</commit_message>
<xml_diff>
--- a/data/final/bplan_samples/annotation/filled_company_templates/test_filled_annotation.xlsx
+++ b/data/final/bplan_samples/annotation/filled_company_templates/test_filled_annotation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>id</t>
   </si>
@@ -62,69 +62,6 @@
   </si>
   <si>
     <t>No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">filename</t>
-  </si>
-  <si>
-    <t xml:space="preserve">met</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">695_0.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grz_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gfz_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eg_fok_value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eg_fok_unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eg_fok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">807_0.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_0.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_1.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_2.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_3.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_4.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_5.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_6.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_7.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">904_8.jpg</t>
   </si>
 </sst>
 </file>
@@ -477,16 +414,16 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="5" t="s">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>4</v>
@@ -500,15 +437,9 @@
       <c r="H1" s="1"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="2" t="n">
-        <v>695</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -516,15 +447,9 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="2" t="n">
-        <v>695</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -532,15 +457,9 @@
       <c r="H3" s="1"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>695</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -548,15 +467,9 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="2" t="n">
-        <v>695</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -564,15 +477,9 @@
       <c r="H5" s="1"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>695</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -580,15 +487,9 @@
       <c r="H6" s="1"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>695</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -596,51 +497,29 @@
       <c r="H7" s="1"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>807</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>0.6</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="4"/>
       <c r="H8" s="1"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="2" t="n">
-        <v>807</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="4"/>
       <c r="H9" s="1"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>807</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -648,15 +527,9 @@
       <c r="H10" s="1"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="2" t="n">
-        <v>807</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -664,15 +537,9 @@
       <c r="H11" s="1"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="2" t="n">
-        <v>807</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -680,15 +547,9 @@
       <c r="H12" s="1"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="2" t="n">
-        <v>807</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -696,51 +557,29 @@
       <c r="H13" s="1"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>0.6</v>
-      </c>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="4"/>
       <c r="H14" s="1"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="4"/>
       <c r="H15" s="1"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -748,15 +587,9 @@
       <c r="H16" s="1"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -764,15 +597,9 @@
       <c r="H17" s="1"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -780,15 +607,9 @@
       <c r="H18" s="1"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -796,15 +617,9 @@
       <c r="H19" s="1"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -812,15 +627,9 @@
       <c r="H20" s="1"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -828,15 +637,9 @@
       <c r="H21" s="1"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -844,15 +647,9 @@
       <c r="H22" s="1"/>
     </row>
     <row r="23" ht="12.5" customHeight="1">
-      <c r="A23" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -860,15 +657,9 @@
       <c r="H23" s="1"/>
     </row>
     <row r="24" ht="12.5" customHeight="1">
-      <c r="A24" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -876,15 +667,9 @@
       <c r="H24" s="1"/>
     </row>
     <row r="25" ht="12.5" customHeight="1">
-      <c r="A25" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -892,15 +677,9 @@
       <c r="H25" s="1"/>
     </row>
     <row r="26" ht="12.5" customHeight="1">
-      <c r="A26" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -908,15 +687,9 @@
       <c r="H26" s="1"/>
     </row>
     <row r="27" ht="12.5" customHeight="1">
-      <c r="A27" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
@@ -924,15 +697,9 @@
       <c r="H27" s="1"/>
     </row>
     <row r="28" ht="12.5" customHeight="1">
-      <c r="A28" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
@@ -940,15 +707,9 @@
       <c r="H28" s="1"/>
     </row>
     <row r="29" ht="12.5" customHeight="1">
-      <c r="A29" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
@@ -956,15 +717,9 @@
       <c r="H29" s="1"/>
     </row>
     <row r="30" ht="12.5" customHeight="1">
-      <c r="A30" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
@@ -972,15 +727,9 @@
       <c r="H30" s="1"/>
     </row>
     <row r="31" ht="12.5" customHeight="1">
-      <c r="A31" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -988,15 +737,9 @@
       <c r="H31" s="1"/>
     </row>
     <row r="32" ht="12.5" customHeight="1">
-      <c r="A32" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
       <c r="D32" s="2"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -1004,15 +747,9 @@
       <c r="H32" s="1"/>
     </row>
     <row r="33" ht="12.5" customHeight="1">
-      <c r="A33" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
@@ -1020,15 +757,9 @@
       <c r="H33" s="1"/>
     </row>
     <row r="34" ht="12.5" customHeight="1">
-      <c r="A34" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -1036,15 +767,9 @@
       <c r="H34" s="1"/>
     </row>
     <row r="35" ht="12.5" customHeight="1">
-      <c r="A35" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
@@ -1052,15 +777,9 @@
       <c r="H35" s="1"/>
     </row>
     <row r="36" ht="12.5" customHeight="1">
-      <c r="A36" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -1068,15 +787,9 @@
       <c r="H36" s="1"/>
     </row>
     <row r="37" ht="12.5" customHeight="1">
-      <c r="A37" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -1084,51 +797,29 @@
       <c r="H37" s="1"/>
     </row>
     <row r="38" ht="12.5" customHeight="1">
-      <c r="A38" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D38" s="2" t="n">
-        <v>0.6</v>
-      </c>
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
       <c r="G38" s="4"/>
       <c r="H38" s="1"/>
     </row>
     <row r="39" ht="12.5" customHeight="1">
-      <c r="A39" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D39" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
       <c r="G39" s="4"/>
       <c r="H39" s="1"/>
     </row>
     <row r="40" ht="12.5" customHeight="1">
-      <c r="A40" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -1136,15 +827,9 @@
       <c r="H40" s="1"/>
     </row>
     <row r="41" ht="12.5" customHeight="1">
-      <c r="A41" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -1152,15 +837,9 @@
       <c r="H41" s="1"/>
     </row>
     <row r="42" ht="12.5" customHeight="1">
-      <c r="A42" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
@@ -1168,15 +847,9 @@
       <c r="H42" s="1"/>
     </row>
     <row r="43" ht="12.5" customHeight="1">
-      <c r="A43" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -1184,15 +857,9 @@
       <c r="H43" s="1"/>
     </row>
     <row r="44" ht="12.5" customHeight="1">
-      <c r="A44" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
@@ -1200,15 +867,9 @@
       <c r="H44" s="1"/>
     </row>
     <row r="45" ht="12.5" customHeight="1">
-      <c r="A45" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
@@ -1216,15 +877,9 @@
       <c r="H45" s="1"/>
     </row>
     <row r="46" ht="12.5" customHeight="1">
-      <c r="A46" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
@@ -1232,15 +887,9 @@
       <c r="H46" s="1"/>
     </row>
     <row r="47" ht="12.5" customHeight="1">
-      <c r="A47" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
@@ -1248,15 +897,9 @@
       <c r="H47" s="1"/>
     </row>
     <row r="48" ht="12.5" customHeight="1">
-      <c r="A48" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
@@ -1264,15 +907,9 @@
       <c r="H48" s="1"/>
     </row>
     <row r="49" ht="12.5" customHeight="1">
-      <c r="A49" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
@@ -1280,15 +917,9 @@
       <c r="H49" s="1"/>
     </row>
     <row r="50" ht="12.5" customHeight="1">
-      <c r="A50" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -1296,15 +927,9 @@
       <c r="H50" s="1"/>
     </row>
     <row r="51" ht="12.5" customHeight="1">
-      <c r="A51" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A51" s="2"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -1312,15 +937,9 @@
       <c r="H51" s="1"/>
     </row>
     <row r="52" ht="12.5" customHeight="1">
-      <c r="A52" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
@@ -1328,15 +947,9 @@
       <c r="H52" s="1"/>
     </row>
     <row r="53" ht="12.5" customHeight="1">
-      <c r="A53" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A53" s="2"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -1344,15 +957,9 @@
       <c r="H53" s="1"/>
     </row>
     <row r="54" ht="12.5" customHeight="1">
-      <c r="A54" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
@@ -1360,15 +967,9 @@
       <c r="H54" s="1"/>
     </row>
     <row r="55" ht="12.5" customHeight="1">
-      <c r="A55" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
       <c r="D55" s="2"/>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
@@ -1376,15 +977,9 @@
       <c r="H55" s="1"/>
     </row>
     <row r="56" ht="12.5" customHeight="1">
-      <c r="A56" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
       <c r="D56" s="2"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
@@ -1392,15 +987,9 @@
       <c r="H56" s="1"/>
     </row>
     <row r="57" ht="12.5" customHeight="1">
-      <c r="A57" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
@@ -1408,15 +997,9 @@
       <c r="H57" s="1"/>
     </row>
     <row r="58" ht="12.5" customHeight="1">
-      <c r="A58" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
@@ -1424,15 +1007,9 @@
       <c r="H58" s="1"/>
     </row>
     <row r="59" ht="12.5" customHeight="1">
-      <c r="A59" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
@@ -1440,15 +1017,9 @@
       <c r="H59" s="1"/>
     </row>
     <row r="60" ht="12.5" customHeight="1">
-      <c r="A60" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
@@ -1456,15 +1027,9 @@
       <c r="H60" s="1"/>
     </row>
     <row r="61" ht="12.5" customHeight="1">
-      <c r="A61" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
@@ -1472,15 +1037,9 @@
       <c r="H61" s="1"/>
     </row>
     <row r="62" ht="12.5" customHeight="1">
-      <c r="A62" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>21</v>
-      </c>
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
       <c r="D62" s="2"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
@@ -1488,15 +1047,9 @@
       <c r="H62" s="1"/>
     </row>
     <row r="63" ht="12.5" customHeight="1">
-      <c r="A63" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
       <c r="D63" s="2"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
@@ -1504,15 +1057,9 @@
       <c r="H63" s="1"/>
     </row>
     <row r="64" ht="12.5" customHeight="1">
-      <c r="A64" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
       <c r="D64" s="2"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
@@ -1520,15 +1067,9 @@
       <c r="H64" s="1"/>
     </row>
     <row r="65" ht="12.5" customHeight="1">
-      <c r="A65" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
@@ -1536,15 +1077,9 @@
       <c r="H65" s="1"/>
     </row>
     <row r="66" ht="12.5" customHeight="1">
-      <c r="A66" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
@@ -1552,15 +1087,9 @@
       <c r="H66" s="1"/>
     </row>
     <row r="67" ht="12.5" customHeight="1">
-      <c r="A67" s="2" t="n">
-        <v>904</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>

</xml_diff>